<commit_message>
final version req v1
</commit_message>
<xml_diff>
--- a/outputs/evaluation/CF_M01_req_eval.xlsx
+++ b/outputs/evaluation/CF_M01_req_eval.xlsx
@@ -492,7 +492,7 @@
         <v>0.8387</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6706</v>
+        <v>0.7238</v>
       </c>
     </row>
     <row r="5">
@@ -520,10 +520,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -538,10 +538,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8667</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8667</v>
+        <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
         <v>26</v>
@@ -760,13 +760,13 @@
         <v>17</v>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" t="n">
         <v>26</v>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.3845</v>
+        <v>0.3751</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>That the system saves the actions carried out on the platform</t>
+          <t>System saves the actions carried out on the platform</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
@@ -1038,16 +1038,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>R_09</t>
+          <t>R_03</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CF_M01_R09</t>
+          <t>CF_M01_R03</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.3852</v>
+        <v>0.4443</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The system shall allow authorized users to list the playlogs.</t>
+          <t>The system shall store the connections of the players.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -1074,11 +1074,11 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Be able to list the different playlogs of the system</t>
+          <t>System saves player connections</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
@@ -1098,7 +1098,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.4262</v>
+        <v>0.4656</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>The actions that the user will be able to see will depend on the permissions what does it have</t>
+          <t>The actions that the user will be able to see will depend on the permissions it has</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
@@ -1148,16 +1148,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>R_29</t>
+          <t>R_13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CF_M01_R27</t>
+          <t>CF_M01_R13</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.4378</v>
+        <v>0.4828</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1166,19 +1166,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Users shall only be able to observe confidential data belonging to their own user account.</t>
+          <t>The connections visible to the user shall depend on their assigned permissions.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>R_28</t>
+          <t>R_12</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -1188,18 +1188,18 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Users can only view their confidential data user and no one else.</t>
+          <t>The connections that the user will be able to see will depend on the permissions it has.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>CF_M01_R026</t>
+          <t>CF_M01_R12</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -1207,67 +1207,75 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>R_12</t>
+          <t>R_29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CF_M01_R12</t>
+          <t>CF_M01_R27</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.4381</v>
+        <v>0.4865</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>criterion</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>39</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>The system shall allow authorized users to list the connections of the players.</t>
+          <t>Users shall only be able to observe the confidential data of their own user account.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>R_28</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>Criterion</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Be able to list the different player connections in the system</t>
+          <t>Users can only view their confidential data user and no one else.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>CF_M01_R026</t>
+        </is>
+      </c>
       <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>R_27</t>
+          <t>R_10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CF_M01_R25</t>
+          <t>CF_M01_R10</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.4609</v>
+        <v>0.4891</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1276,19 +1284,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Users without permission shall not be able to access data for which they do not have authorization.</t>
+          <t>The playlogs visible to the user shall depend on their assigned permissions.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>R_26</t>
+          <t>R_09</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -1298,18 +1306,18 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Unauthorized users cannot access data they do not own.</t>
+          <t>The playlogs that the user will be able to see will depend on the permissions it has</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>CF_M01_R024</t>
+          <t>CF_M01_R09</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -1317,16 +1325,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>R_03</t>
+          <t>R_15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CF_M01_R03</t>
+          <t>CF_M01_R15</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.4742</v>
+        <v>0.5417999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1335,12 +1343,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>37</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>The system shall store the connections of the players.</t>
+          <t>The system shall allow users with permissions to list the different actions performed on the platform entities.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1353,11 +1361,12 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Let the system save player connections</t>
+          <t>Be able to list the different actions that are carried out on the different
+platform entities</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -1368,134 +1377,134 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R_13</t>
+          <t>R_01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CF_M01_R13</t>
+          <t>CF_M01_R01</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.4808</v>
+        <v>0.543</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>criterion</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>The connections visible to the user shall depend on their assigned permissions.</t>
+          <t>The system shall store the playlogs of the players.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>R_12</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Criterion</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>The connections that the user will be able to see will depend on the permissions you have.</t>
+          <t>System saves the players' playlogs</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>CF_M01_R12</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R_10</t>
+          <t>R_20</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CF_M01_R10</t>
+          <t>CF_M01_R20</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.4999</v>
+        <v>0.5964</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>The playlogs visible to the user shall depend on their assigned permissions.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>R_09</t>
-        </is>
-      </c>
+          <t>The system must be available at all times, except for scheduled updates.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Availability and reliability</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>The playlogs that the user will be able to see will depend on the permissions it has</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>CF_M01_R09</t>
-        </is>
-      </c>
+          <t>The system must be available at all times, except for some punctuality, such as an update.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>12d. Availability and reliability</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>R_01</t>
+          <t>R_12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CF_M01_R01</t>
+          <t>CF_M01_R12</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.5523</v>
+        <v>0.6706</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1504,12 +1513,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>The system shall store the playlogs of the players.</t>
+          <t>The system shall allow users with permissions to list the different connections of the players in the system.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1522,11 +1531,11 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>That the system saves the players' playlogs</t>
+          <t>Be able to list the different player connections in the system</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
@@ -1537,83 +1546,67 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>R_20</t>
+          <t>R_09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CF_M01_R20</t>
+          <t>CF_M01_R09</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.5756</v>
+        <v>0.6864</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>The system shall be available at all times, except for scheduled updates.</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Availability and reliability</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>ISO/IEC 25010</t>
-        </is>
-      </c>
+          <t>The system shall allow users with permissions to list the different playlogs of the system.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="L12" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>The system must be available at all times, except for some punctuality, such as an update.</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>12d. Availability and reliability</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Volere</t>
-        </is>
-      </c>
+          <t>Be able to list the different playlogs of the system</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>R_22</t>
+          <t>R_28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CF_M01_R22</t>
+          <t>CF_M01_R26</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.6114000000000001</v>
+        <v>0.7096</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1622,22 +1615,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>The system shall be capable of supporting an unlimited number of concurrent connections.</t>
+          <t>Confidential user information must be protected to ensure privacy.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>ISO/IEC 25010</t>
+          <t>Volere</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1648,17 +1641,17 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>The system must be able to support an unlimited number of
-connections at the same time.</t>
+          <t>Users' confidential information must be protected in order to
+guarantee your privacy.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>12f. Capacity</t>
+          <t>15c. Privacy</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1672,16 +1665,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R_07</t>
+          <t>R_08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CF_M01_R07</t>
+          <t>CF_M01_R08</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.6679</v>
+        <v>0.7406</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1695,7 +1688,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Each action must have a date, client, user, and player assigned.</t>
+          <t>All actions must be performed on a platform entity.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1716,7 +1709,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Each action has an assigned date, client and player.</t>
+          <t>All actions are performed on an entity of the platform.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr"/>
@@ -1731,84 +1724,75 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R_28</t>
+          <t>R_07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CF_M01_R26</t>
+          <t>CF_M01_R07</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.7124</v>
+        <v>0.7759</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>criterion</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Confidential user information must be protected to ensure privacy.</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>ISO/IEC 25010</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>Each action must have a date, client, user, and assigned player.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>R_06</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>Criterion</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Users' confidential information must be protected in order to
-guarantee your privacy.</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>15c. Privacy</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Volere</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
+          <t>Each action has an assigned date, client and player.</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>CF_M01_R06</t>
+        </is>
+      </c>
       <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>R_04</t>
+          <t>R_17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CF_M01_R04</t>
+          <t>CF_M01_R17</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.763</v>
+        <v>0.8153</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1817,19 +1801,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>37</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Each connection must have a date, client, and player assigned.</t>
+          <t>All actions must be related to a platform entity.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>R_03</t>
+          <t>R_15</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1839,18 +1823,18 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Each connection has an assigned date, client, player.</t>
+          <t>All actions must be related to an entity the platform.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>CF_M01_R03</t>
+          <t>CF_M01_R015</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr"/>
@@ -1858,16 +1842,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R_02</t>
+          <t>R_04</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CF_M01_R02</t>
+          <t>CF_M01_R04</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.7766</v>
+        <v>0.8748</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1881,14 +1865,14 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Each playlog must have a date, client, and player assigned.</t>
+          <t>Each connection must have a date, client, and assigned player.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>R_01</t>
+          <t>R_03</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1902,14 +1886,14 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Each playlog has an assigned date, client, player.</t>
+          <t>Each connection has an assigned date, client, player.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>CF_M01_R01</t>
+          <t>CF_M01_R03</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -1917,16 +1901,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>R_11</t>
+          <t>R_02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CF_M01_R11</t>
+          <t>CF_M01_R02</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.7966</v>
+        <v>0.8821</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1935,19 +1919,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>35</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>The user must be able to view all details of the playlog.</t>
+          <t>Each playlog must have a date, client, and assigned player.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>R_09</t>
+          <t>R_01</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1957,18 +1941,18 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>You must be able to see all the details of the playlog.</t>
+          <t>Each playlog has an assigned date, client, player.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>CF_M01_R09</t>
+          <t>CF_M01_R01</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -1976,84 +1960,75 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>R_26</t>
+          <t>R_19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CF_M01_R24</t>
+          <t>CF_M01_R19</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.8642</v>
+        <v>0.907</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>criterion</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>37</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>System functionalities shall only be accessible to users with the corresponding permissions.</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Access</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>ISO/IEC 25010</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
+          <t>The system shall respond to any user action in less than 5 seconds.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>R_18</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>Criterion</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>The project's functionalities must only be accessible to
-users with the corresponding permissions.</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>15a. Access</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Volere</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr"/>
+          <t>The system responds to any user action in less than 5 seconds.</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>CF_M01_R018</t>
+        </is>
+      </c>
       <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R_19</t>
+          <t>R_11</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CF_M01_R19</t>
+          <t>CF_M01_R11</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.9135</v>
+        <v>0.9115</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2062,19 +2037,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>The system shall respond to any user action in less than 5 seconds.</t>
+          <t>The user must be able to see all details of the playlog.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>R_18</t>
+          <t>R_09</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -2084,18 +2059,18 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>The system responds to any user action in less than 5 seconds.</t>
+          <t>You must be able to see all the details of the playlog.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>CF_M01_R018</t>
+          <t>CF_M01_R09</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr"/>
@@ -2103,265 +2078,267 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R_18</t>
+          <t>R_21</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CF_M01_R18</t>
+          <t>CF_M01_R21</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.931</v>
+        <v>0.9352</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>criterion</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>The system shall respond quickly when the user performs an action.</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Speed and latency</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>ISO/IEC 25010</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>Any user must be able to access the platform at any time of the day, except during scheduled updates.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>R_20</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>Criterion</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>The system must respond quickly when the user performs any action.</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>12a. Speed and latency</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>Volere</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr"/>
+          <t>Any user must be able to access the platform during any time
+time of day. Except for scheduled updates.</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>CF_M01_R020</t>
+        </is>
+      </c>
       <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>R_21</t>
+          <t>R_26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CF_M01_R21</t>
+          <t>CF_M01_R24</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.9343</v>
+        <v>1</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Any user must be able to access the platform at any time of the day, except during scheduled updates.</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>R_20</t>
-        </is>
-      </c>
+          <t>The project functionalities must only be accessible to users with the corresponding permissions.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Access</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Any user must be able to access the platform during any time
-time of day. Except for scheduled updates.</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>CF_M01_R020</t>
-        </is>
-      </c>
+          <t>The project's functionalities must only be accessible to
+users with the corresponding permissions.</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>15a. Access</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R_24</t>
+          <t>R_14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CF_M01_R23</t>
+          <t>CF_M01_R14</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.9462</v>
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>criterion</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>36</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>The system shall be able to grow in capacity when the volume of data increases.</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Scalability</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>ISO/IEC 25010</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>Connections can only have two states: connected or not connected.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>R_12</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>QR</t>
+          <t>Criterion</t>
         </is>
       </c>
       <c r="L23" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>The system must be able to grow in capacity as the volume of data increases.</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>12g. Scalability</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Volere</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr"/>
+          <t>Connections can only have two states: connected or not connected.</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>CF_M01_R12</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R_14</t>
+          <t>R_22</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CF_M01_R14</t>
+          <t>CF_M01_R22</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.9674</v>
+        <v>1</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Connections shall only have two states: connected or not connected.</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>R_12</t>
-        </is>
-      </c>
+          <t>The system must be able to support an unlimited number of connections at the same time.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Connections can only have two states: connected or not connected.</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>CF_M01_R12</t>
-        </is>
-      </c>
+          <t>The system must be able to support an unlimited number of
+connections at the same time.</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>12f. Capacity</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>R_17</t>
+          <t>R_24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CF_M01_R17</t>
+          <t>CF_M01_R23</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -2369,58 +2346,66 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>All actions must be related to an entity of the platform.</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>R_15</t>
-        </is>
-      </c>
+          <t>The system must be able to grow in capacity when the volume of data increases.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Scalability</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>All actions must be related to an entity the platform.</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>CF_M01_R015</t>
-        </is>
-      </c>
+          <t>The system must be able to grow in capacity as the volume of data increases.</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>12g. Scalability</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R_08</t>
+          <t>R_18</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CF_M01_R08</t>
+          <t>CF_M01_R18</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -2428,47 +2413,55 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>All actions must be performed on an entity of the platform.</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>R_06</t>
-        </is>
-      </c>
+          <t>The system must respond quickly when the user performs any action.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Speed and latency</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Criterion</t>
+          <t>QR</t>
         </is>
       </c>
       <c r="L26" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>All actions are performed on an entity of the platform.</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>CF_M01_R06</t>
-        </is>
-      </c>
+          <t>The system must respond quickly when the user performs any action.</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>12a. Speed and latency</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Volere</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -2579,37 +2572,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>R_15</t>
+          <t>R_23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>criterion</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The system shall allow authorized users to list the actions performed on the platform entities.</t>
+          <t>The platform shall scale dynamically with changes in simultaneous connections.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CF_M01_R08</t>
+          <t>CF_M01_R05</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>All actions are performed on an entity of the platform.</t>
+          <t>The connection status can only be connected or not connected.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.5184</v>
+        <v>0.1564</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>R_23</t>
+          <t>R_25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2619,27 +2612,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The platform shall scale dynamically with changes in simultaneous connections.</t>
+          <t>The system shall scale automatically as data increases.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CF_M01_R05</t>
+          <t>CF_M01_R23</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The connection status can only be connected or not connected.</t>
+          <t>The system must be able to grow in capacity as the volume of data increases.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.156</v>
+        <v>0.3857</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>R_25</t>
+          <t>R_27</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2649,21 +2642,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The system shall scale automatically as data increases.</t>
+          <t>Users without permission shall not be able to access data for which they do not have permission.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CF_M01_R23</t>
+          <t>CF_M01_R25</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The system must be able to grow in capacity as the volume of data increases.</t>
+          <t>Unauthorized users cannot access data they do not own.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.3909</v>
+        <v>0.3483</v>
       </c>
     </row>
   </sheetData>
@@ -2715,32 +2708,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CF_M01_R15</t>
+          <t>CF_M01_R25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>Criterion</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Be able to list the different actions that are carried out on the different
-platform entities</t>
+          <t>Unauthorized users cannot access data they do not own.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>R_15</t>
+          <t>R_27</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>The system shall allow authorized users to list the actions performed on the platform entities.</t>
+          <t>Users without permission shall not be able to access data for which they do not have permission.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.326</v>
+        <v>0.3483</v>
       </c>
     </row>
     <row r="3">
@@ -2761,16 +2753,16 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>R_07</t>
+          <t>R_09</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Each action must have a date, client, user, and player assigned.</t>
+          <t>The system shall allow users with permissions to list the different playlogs of the system.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.1132</v>
+        <v>0.2428</v>
       </c>
     </row>
     <row r="4">
@@ -2800,7 +2792,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.3212</v>
+        <v>0.3222</v>
       </c>
     </row>
     <row r="5">
@@ -2826,11 +2818,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The system shall allow authorized users to list the connections of the players.</t>
+          <t>The system shall allow users with permissions to list the different connections of the players in the system.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.1579</v>
+        <v>0.2979</v>
       </c>
     </row>
     <row r="6">
@@ -2860,7 +2852,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.2956</v>
+        <v>0.2963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>